<commit_message>
scalebay update 2026-07-05 01:12 (1923 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -824,67 +824,6 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Skoda 706 RTTN с полуприцепом Alka N12CH   АИСТ</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-2.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-3.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-8.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-9.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-6.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-7.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-5.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-10.jpg</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>7409184</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>4100</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Škoda</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Автоистория (АИСТ)</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>металл , пластик, резина</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>Информация по оплате и отправке в разделе " Обо мне". Условия аукциона стандартные. выход на связь в течении 3 дней оплата в течении 7 дней с момента окончания аукциона. Все вопросы по лоту , оплате , отправке исключительно до покупки (до ставки) Смотрите мои другие лоты.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-06 01:31 (1885 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -824,6 +824,67 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Skoda 706 RTTN с полуприцепом Alka N12CH   АИСТ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-2.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-3.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-8.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-9.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-6.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-7.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-5.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-10.jpg</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>7409184</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>4100</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="n">
+        <v>4100</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Škoda</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Автоистория (АИСТ)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>металл , пластик, резина</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Новый</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Информация по оплате и отправке в разделе " Обо мне". Условия аукциона стандартные. выход на связь в течении 3 дней оплата в течении 7 дней с момента окончания аукциона. Все вопросы по лоту , оплате , отправке исключительно до покупки (до ставки) Смотрите мои другие лоты.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-06 13:40 (2033 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -598,17 +598,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mercedes Brabus 850 6.0 Widestar  2016 Minichamps</t>
+          <t>Mercedes Brabus G  V12 Widestar 2010  Minichamps</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134535.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134448.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134541.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134547.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134601.jpg</t>
+          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175143.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175106.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175136.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175148.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175203.jpg</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>4213802</t>
+          <t>7151583</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>Brabus</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -657,22 +657,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Mercedes Brabus G  V12 Widestar 2010  Minichamps</t>
+          <t>Mercedes C-Klasse 2011 W204 W 204 Schuco</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175143.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175106.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175136.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175148.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175203.jpg</t>
+          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135744.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135654.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135703.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135716.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135721.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135755.jpg</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>7151583</t>
+          <t>7830441</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>9200</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -680,16 +680,16 @@
         <v>300</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>9500</v>
+        <v>9300</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Brabus</t>
+          <t>Mercedes-Benz</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Minichamps</t>
+          <t>Schuco</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Отправляю по всему миру - по возможности.</t>
+          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкойПривезу любые модели на заказ.</t>
         </is>
       </c>
     </row>
@@ -716,22 +716,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Mercedes C-Klasse 2011 W204 W 204 Schuco</t>
+          <t>Audi RS4 RS 4 Avant  2018 Spark</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135744.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135654.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135703.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135716.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135721.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135755.jpg</t>
+          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471219.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471242.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471236.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471229.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471223.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471213.jpg</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>7830441</t>
+          <t>9331546</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>9300</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -739,33 +739,29 @@
         <v>300</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>9300</v>
+        <v>9600</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>Audi</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Schuco</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
+          <t>Spark</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Б/у</t>
+          <t>Новый</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкойПривезу любые модели на заказ.</t>
+          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Привезу любые модели на заказ.</t>
         </is>
       </c>
     </row>
@@ -775,43 +771,49 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Audi RS4 RS 4 Avant  2018 Spark</t>
+          <t>Skoda 706 RTTN с полуприцепом Alka N12CH   АИСТ</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471219.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471242.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471236.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471229.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471223.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471213.jpg</t>
+          <t>https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-2.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-3.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-8.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-9.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-6.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-7.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-5.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-10.jpg</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>9331546</t>
+          <t>7409184</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>9300</t>
+          <t>4100</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="n">
-        <v>300</v>
-      </c>
+      <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="n">
-        <v>9600</v>
+        <v>4100</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Audi</t>
+          <t>Škoda</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Spark</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+          <t>Автоистория (АИСТ)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>металл , пластик, резина</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -819,67 +821,6 @@
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Привезу любые модели на заказ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Skoda 706 RTTN с полуприцепом Alka N12CH   АИСТ</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-2.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-3.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-8.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-9.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-6.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-7.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-5.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-10.jpg</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>7409184</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>4100</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Škoda</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Автоистория (АИСТ)</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>металл , пластик, резина</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Информация по оплате и отправке в разделе " Обо мне". Условия аукциона стандартные. выход на связь в течении 3 дней оплата в течении 7 дней с момента окончания аукциона. Все вопросы по лоту , оплате , отправке исключительно до покупки (до ставки) Смотрите мои другие лоты.</t>
         </is>

</xml_diff>

<commit_message>
scalebay update 2026-07-08 10:07 (1934 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,13 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,299 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Chevrolet Camaro Rally Sport 1978 Neo</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/1734018782485.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1734018782499.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1734018782496.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1734018782493.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1734018782489.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>4134455</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>9200</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>9500</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Chevrolet</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Neo Scale Models</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Б/у</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Привезу любые модели на заказ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Mercedes Brabus G  V12 Widestar 2010  Minichamps</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175143.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175106.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175136.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175148.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175203.jpg</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>7151583</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>9200</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>9500</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Brabus</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Minichamps</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Б/у</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Отправляю по всему миру - по возможности.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Mercedes C-Klasse 2011 W204 W 204 Schuco</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135744.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135654.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135703.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135716.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135721.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251123_135755.jpg</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>7830441</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>9000</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>9300</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Schuco</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Б/у</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкойПривезу любые модели на заказ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Audi RS4 RS 4 Avant  2018 Spark</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471219.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471242.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471236.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471229.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471223.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471213.jpg</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>9331546</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>9300</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>9600</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Spark</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Привезу любые модели на заказ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Skoda 706 RTTN с полуприцепом Alka N12CH   АИСТ</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-2.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-3.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-8.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-9.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-6.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-7.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-5.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-10.jpg</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>7409184</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>4100</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
-        <v>4100</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Škoda</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Автоистория (АИСТ)</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>металл , пластик, резина</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>Информация по оплате и отправке в разделе " Обо мне". Условия аукциона стандартные. выход на связь в течении 3 дней оплата в течении 7 дней с момента окончания аукциона. Все вопросы по лоту , оплате , отправке исключительно до покупки (до ставки) Смотрите мои другие лоты.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-09 10:30 (2199 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -530,6 +533,55 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BERLIET 560K, grey</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1518816</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Berliet</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Altaya</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-09 12:36 (2192 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,13 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,55 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>BERLIET 560K, grey</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>1518816</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
-        <v>1950</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Berliet</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Altaya</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-09 14:44 (2200 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -530,6 +533,55 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BERLIET 560K, grey</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1518816</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Berliet</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Altaya</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-10 02:56 (2185 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,13 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,55 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>BERLIET 560K, grey</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>1518816</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
-        <v>1950</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Berliet</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Altaya</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-10 15:06 (2059 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -530,6 +533,55 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BERLIET 560K, grey</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1518816</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Berliet</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Altaya</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-11 03:18 (1963 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,13 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,55 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>BERLIET 560K, grey</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>1518816</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
-        <v>1950</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Berliet</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Altaya</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-11 15:28 (2050 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -530,6 +533,55 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BERLIET 560K, grey</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1518816</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Berliet</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Altaya</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-12 03:39 (2188 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,13 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,55 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>BERLIET 560K, grey</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>1518816</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1950</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
-        <v>1950</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Berliet</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Altaya</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-12 15:49 (2073 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -530,6 +533,55 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BERLIET 560K, grey</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/v/d/vdim_1858/1-8-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1518816</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1950</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n">
+        <v>1950</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Berliet</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Altaya</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-16 20:57 (6076 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,13 +63,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,411 +530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Камаз-6520 рестайлинг самосвал.SSM.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/cache/user/a/r/artmodel_31719/11-16-213x128.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>869462</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>8500</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>8550</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>КамАЗ</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Start Scale Models (SSM)</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Porsche 911 Dakar 2023</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/m/a/mandiby_7644/20240517_150958.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20240517_150925.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20240517_150950.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20240517_151006.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20240517_151020.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20240517_151014.jpg</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>1391757</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>9198</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>9498</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Porsche</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Minichamps</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>Модель абсолютно новая.доставалась из коробки только для фотографирования.При отправке почтой,гарантирую надежную упаковку.Возможно объединение нескольких лотов. Отвечу на все Ваши вопросы (до покупки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Mercedes X-Class 2017</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/m/a/mandiby_7644/mercedes-x-klasse-norev-183421-6.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202209.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202532.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202227.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202414.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202238.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202319.jpg</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>4439325</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>9298</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>9598</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Norev</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>1:18</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>Модель абсолютно новая.доставалась из коробки только для фотографирования.При отправке почтой,гарантирую надежную упаковку.Возможно объединение нескольких лотов. Отвечу на все Ваши вопросы (до покупки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Audi RS e-tron GT 2021 anthrazit</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/m/a/mandiby_7644/20211008_195304.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/89939.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/89939r.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20211008_195227.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20211008_195337.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20211008_195318.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20211008_195327.jpg</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>5884616</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>9298</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>9598</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Norev</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>1:18</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>Модель абсолютно новая.доставалась из коробки только для фотографирования.При отправке почтой,гарантирую надежную упаковку.Возможно объединение нескольких лотов. Отвечу на все Ваши вопросы (до покупки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen Hebmüller Cabriolet 1950</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102927-(1).jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102845-(1).jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102850-(1).jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102910-(1).jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102919-(1).jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102923-(1).jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20250421_102931-(1).jpg</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>7850859</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>4398</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>4698</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Volkswagen</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Minichamps</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>Модель абсолютно новая.доставалась из коробки только для фотографирования.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>КамАЗ-6522 самосвал белый</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-2.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-1.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-4.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-3.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-7.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-5.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-8.jpg</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>1613562</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>3900</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>4200</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>КамАЗ</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>ПАО КАМАЗ</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Металл/пластмасса</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>104165</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>Модель новая в оригинальной упаковке.Самовывоз в Москве от метро Строгино.Почта России или СДЭК от 500 рублей.Выход на связь 1 день, оплата на карту Альфа банка 5 дней.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>ДЭ-210 (ЗиЛ-131)</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/cache/user/a/v/avtobusnik_6320/de-210-131-663854-2-213x128.jpg</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>9580455</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>5750</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>6050</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>ЗИЛ</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Start Scale Models (SSM)</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-07-16 21:24 (6185 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -63,10 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -530,6 +533,516 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr L 586 NZG</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_155721-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1125819</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>17000</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>17300</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>NZG</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr PR 776 бульдозер WSI</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_151010-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1151941</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>25000</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>25300</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>WSI</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr T 264 самосвал Conrad</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_165051-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1291831</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>40000</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>40300</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Conrad</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr R 9400 NZG</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_153515-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2960452</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>45000</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>45300</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>NZG</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель БТР-60 ПБ СССР</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20241221_231012-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>4107794</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>3500</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>3800</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>БТР</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Арсенал</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr PR 754 NZG</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_144742-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>4281382</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>12000</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>12300</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>NZG</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr R 9800 NZG</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_172802-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>4335434</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>75000</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>75300</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>NZG</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr PR 764 NZG</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_145952-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>5764964</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>15300</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>NZG</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr R 9100 экскаватор Conrad</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_164242-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>5799020</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>32000</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>32300</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Conrad</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Масштабная модель Liebherr TA 230 Conrad</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/cache/user/n/i/nik6001_303/img_20250211_145304-213x128.jpg</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>9613326</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>15300</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Conrad</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>1:50</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scalebay update 2026-08-21 05:44 (6301 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дальние" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Дальние" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
scalebay update 2026-08-21 06:15 (6335 lots)
</commit_message>
<xml_diff>
--- a/scalebay_latest_far.xlsx
+++ b/scalebay_latest_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Дальние" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дальние" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>